<commit_message>
FacilityData 컬럼 추가. Drill1 추가
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
@@ -121,7 +121,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -195,7 +195,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -302,7 +302,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="85">
   <si>
     <t>0,0</t>
   </si>
@@ -577,6 +577,33 @@
   </si>
   <si>
     <t>laboratory5</t>
+  </si>
+  <si>
+    <t>ActionClassName</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>HelloFacilityAction</t>
+  </si>
+  <si>
+    <t>drill1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>드릴 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Drill</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0;0,1;</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>DrillAction</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1260,14 +1287,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="표2" displayName="표2" ref="A1:L29" totalsRowShown="0">
-  <autoFilter ref="A1:L29"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="표2" displayName="표2" ref="A1:M30" totalsRowShown="0">
+  <autoFilter ref="A1:M30"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="5" name="Name"/>
     <tableColumn id="2" name="DisplayName"/>
     <tableColumn id="8" name="Type"/>
     <tableColumn id="3" name="Level"/>
+    <tableColumn id="13" name="ActionClassName"/>
     <tableColumn id="11" name="BuildResourceId"/>
     <tableColumn id="12" name="BuildResourceCount"/>
     <tableColumn id="7" name="InputItemId"/>
@@ -1543,7 +1571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.25" customWidth="1"/>
@@ -1555,7 +1583,7 @@
     <col min="12" max="12" width="18.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1572,28 +1600,31 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" t="s">
         <v>47</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>48</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>23</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>101011</v>
       </c>
@@ -1609,17 +1640,20 @@
       <c r="E2">
         <v>1</v>
       </c>
-      <c r="J2">
+      <c r="F2" t="s">
+        <v>79</v>
+      </c>
+      <c r="K2">
         <v>1001</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>1</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>101012</v>
       </c>
@@ -1635,17 +1669,20 @@
       <c r="E3">
         <v>2</v>
       </c>
-      <c r="J3">
+      <c r="F3" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3">
         <v>1001</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>10</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>101013</v>
       </c>
@@ -1661,17 +1698,20 @@
       <c r="E4">
         <v>3</v>
       </c>
-      <c r="J4">
+      <c r="F4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K4">
         <v>1001</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>100</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>101021</v>
       </c>
@@ -1687,23 +1727,26 @@
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="H5">
+      <c r="F5" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5">
         <v>1001</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>1</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>1002</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>1</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>101022</v>
       </c>
@@ -1719,23 +1762,26 @@
       <c r="E6">
         <v>2</v>
       </c>
-      <c r="H6">
+      <c r="F6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6">
         <v>1001</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>10</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>1002</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>10</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>101023</v>
       </c>
@@ -1751,23 +1797,26 @@
       <c r="E7">
         <v>3</v>
       </c>
-      <c r="H7">
+      <c r="F7" t="s">
+        <v>79</v>
+      </c>
+      <c r="I7">
         <v>1001</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>100</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>1002</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>100</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>102011</v>
       </c>
@@ -1783,17 +1832,20 @@
       <c r="E8">
         <v>1</v>
       </c>
-      <c r="J8">
+      <c r="F8" t="s">
+        <v>79</v>
+      </c>
+      <c r="K8">
         <v>1003</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>1</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>102012</v>
       </c>
@@ -1809,17 +1861,20 @@
       <c r="E9">
         <v>2</v>
       </c>
-      <c r="J9">
+      <c r="F9" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9">
         <v>1003</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>10</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>102013</v>
       </c>
@@ -1835,17 +1890,20 @@
       <c r="E10">
         <v>3</v>
       </c>
-      <c r="J10">
+      <c r="F10" t="s">
+        <v>79</v>
+      </c>
+      <c r="K10">
         <v>1003</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>100</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>102021</v>
       </c>
@@ -1861,23 +1919,26 @@
       <c r="E11">
         <v>1</v>
       </c>
-      <c r="H11">
+      <c r="F11" t="s">
+        <v>79</v>
+      </c>
+      <c r="I11">
         <v>1003</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>1</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>1004</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>1</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>102022</v>
       </c>
@@ -1893,23 +1954,26 @@
       <c r="E12">
         <v>2</v>
       </c>
-      <c r="H12">
+      <c r="F12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I12">
         <v>1003</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>10</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>1004</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>10</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>102023</v>
       </c>
@@ -1925,23 +1989,26 @@
       <c r="E13">
         <v>3</v>
       </c>
-      <c r="H13">
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="I13">
         <v>1003</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>100</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>1004</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>100</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>103011</v>
       </c>
@@ -1957,17 +2024,20 @@
       <c r="E14">
         <v>1</v>
       </c>
-      <c r="J14">
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K14">
         <v>1005</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>1</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>103012</v>
       </c>
@@ -1983,17 +2053,20 @@
       <c r="E15">
         <v>2</v>
       </c>
-      <c r="J15">
+      <c r="F15" t="s">
+        <v>79</v>
+      </c>
+      <c r="K15">
         <v>1005</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>10</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>103013</v>
       </c>
@@ -2009,17 +2082,20 @@
       <c r="E16">
         <v>3</v>
       </c>
-      <c r="J16">
+      <c r="F16" t="s">
+        <v>79</v>
+      </c>
+      <c r="K16">
         <v>1005</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>100</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>103021</v>
       </c>
@@ -2035,23 +2111,26 @@
       <c r="E17">
         <v>1</v>
       </c>
-      <c r="H17">
+      <c r="F17" t="s">
+        <v>79</v>
+      </c>
+      <c r="I17">
         <v>1004</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>1</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>1006</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>1</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>103022</v>
       </c>
@@ -2067,23 +2146,26 @@
       <c r="E18">
         <v>2</v>
       </c>
-      <c r="H18">
+      <c r="F18" t="s">
+        <v>79</v>
+      </c>
+      <c r="I18">
         <v>1004</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>10</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>1005</v>
       </c>
-      <c r="K18">
+      <c r="L18">
         <v>10</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>103023</v>
       </c>
@@ -2099,23 +2181,26 @@
       <c r="E19">
         <v>3</v>
       </c>
-      <c r="H19">
+      <c r="F19" t="s">
+        <v>79</v>
+      </c>
+      <c r="I19">
         <v>1004</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>100</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>1005</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>100</v>
       </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>110001</v>
       </c>
@@ -2131,11 +2216,14 @@
       <c r="E20">
         <v>1</v>
       </c>
-      <c r="L20" t="s">
+      <c r="F20" t="s">
+        <v>79</v>
+      </c>
+      <c r="M20" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>110002</v>
       </c>
@@ -2151,11 +2239,14 @@
       <c r="E21">
         <v>2</v>
       </c>
-      <c r="L21" t="s">
+      <c r="F21" t="s">
+        <v>79</v>
+      </c>
+      <c r="M21" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>110003</v>
       </c>
@@ -2171,11 +2262,14 @@
       <c r="E22">
         <v>3</v>
       </c>
-      <c r="L22" t="s">
+      <c r="F22" t="s">
+        <v>79</v>
+      </c>
+      <c r="M22" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>110004</v>
       </c>
@@ -2191,11 +2285,14 @@
       <c r="E23">
         <v>4</v>
       </c>
-      <c r="L23" t="s">
+      <c r="F23" t="s">
+        <v>79</v>
+      </c>
+      <c r="M23" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>110005</v>
       </c>
@@ -2211,11 +2308,14 @@
       <c r="E24">
         <v>5</v>
       </c>
-      <c r="L24" t="s">
+      <c r="F24" t="s">
+        <v>79</v>
+      </c>
+      <c r="M24" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>111001</v>
       </c>
@@ -2231,11 +2331,14 @@
       <c r="E25">
         <v>1</v>
       </c>
-      <c r="L25" t="s">
+      <c r="F25" t="s">
+        <v>79</v>
+      </c>
+      <c r="M25" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>111002</v>
       </c>
@@ -2251,11 +2354,14 @@
       <c r="E26">
         <v>2</v>
       </c>
-      <c r="L26" t="s">
+      <c r="F26" t="s">
+        <v>79</v>
+      </c>
+      <c r="M26" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>111003</v>
       </c>
@@ -2271,11 +2377,14 @@
       <c r="E27">
         <v>3</v>
       </c>
-      <c r="L27" t="s">
+      <c r="F27" t="s">
+        <v>79</v>
+      </c>
+      <c r="M27" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>111004</v>
       </c>
@@ -2291,11 +2400,14 @@
       <c r="E28">
         <v>4</v>
       </c>
-      <c r="L28" t="s">
+      <c r="F28" t="s">
+        <v>79</v>
+      </c>
+      <c r="M28" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>111005</v>
       </c>
@@ -2311,8 +2423,34 @@
       <c r="E29">
         <v>5</v>
       </c>
-      <c r="L29" t="s">
+      <c r="F29" t="s">
+        <v>79</v>
+      </c>
+      <c r="M29" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>112001</v>
+      </c>
+      <c r="B30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" t="s">
+        <v>81</v>
+      </c>
+      <c r="D30" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30" t="s">
+        <v>84</v>
+      </c>
+      <c r="M30" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Facility들의 coordinate가 load되지 않던 문제 해결
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
@@ -315,10 +315,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>Coordinate</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>DisplayName</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -603,6 +599,10 @@
   </si>
   <si>
     <t>DrillAction</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Coordinates</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1302,7 +1302,7 @@
     <tableColumn id="10" name="InputItemCount"/>
     <tableColumn id="6" name="OutputItemId"/>
     <tableColumn id="9" name="OutputItemCount"/>
-    <tableColumn id="4" name="Coordinate"/>
+    <tableColumn id="4" name="Coordinates"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1581,6 +1581,7 @@
     <col min="7" max="7" width="22.5" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="12" max="12" width="18.125" customWidth="1"/>
+    <col min="13" max="13" width="17.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
@@ -1588,40 +1589,40 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="H1" t="s">
-        <v>48</v>
-      </c>
       <c r="I1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>22</v>
       </c>
-      <c r="K1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" t="s">
-        <v>23</v>
-      </c>
       <c r="M1" t="s">
-        <v>3</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -1629,19 +1630,19 @@
         <v>101011</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K2">
         <v>1001</v>
@@ -1658,19 +1659,19 @@
         <v>101012</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K3">
         <v>1001</v>
@@ -1679,7 +1680,7 @@
         <v>10</v>
       </c>
       <c r="M3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -1687,19 +1688,19 @@
         <v>101013</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4">
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K4">
         <v>1001</v>
@@ -1708,7 +1709,7 @@
         <v>100</v>
       </c>
       <c r="M4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -1716,19 +1717,19 @@
         <v>101021</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I5">
         <v>1001</v>
@@ -1751,19 +1752,19 @@
         <v>101022</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E6">
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I6">
         <v>1001</v>
@@ -1778,7 +1779,7 @@
         <v>10</v>
       </c>
       <c r="M6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -1786,19 +1787,19 @@
         <v>101023</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I7">
         <v>1001</v>
@@ -1813,7 +1814,7 @@
         <v>100</v>
       </c>
       <c r="M7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -1821,19 +1822,19 @@
         <v>102011</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K8">
         <v>1003</v>
@@ -1850,19 +1851,19 @@
         <v>102012</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9">
         <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K9">
         <v>1003</v>
@@ -1871,7 +1872,7 @@
         <v>10</v>
       </c>
       <c r="M9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -1879,19 +1880,19 @@
         <v>102013</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10">
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K10">
         <v>1003</v>
@@ -1900,7 +1901,7 @@
         <v>100</v>
       </c>
       <c r="M10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -1908,19 +1909,19 @@
         <v>102021</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I11">
         <v>1003</v>
@@ -1943,19 +1944,19 @@
         <v>102022</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12">
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I12">
         <v>1003</v>
@@ -1970,7 +1971,7 @@
         <v>10</v>
       </c>
       <c r="M12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -1978,19 +1979,19 @@
         <v>102023</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13">
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I13">
         <v>1003</v>
@@ -2005,7 +2006,7 @@
         <v>100</v>
       </c>
       <c r="M13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -2013,19 +2014,19 @@
         <v>103011</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K14">
         <v>1005</v>
@@ -2042,19 +2043,19 @@
         <v>103012</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E15">
         <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K15">
         <v>1005</v>
@@ -2063,7 +2064,7 @@
         <v>10</v>
       </c>
       <c r="M15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
@@ -2071,19 +2072,19 @@
         <v>103013</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E16">
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K16">
         <v>1005</v>
@@ -2092,7 +2093,7 @@
         <v>100</v>
       </c>
       <c r="M16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
@@ -2100,19 +2101,19 @@
         <v>103021</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I17">
         <v>1004</v>
@@ -2135,19 +2136,19 @@
         <v>103022</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I18">
         <v>1004</v>
@@ -2162,7 +2163,7 @@
         <v>10</v>
       </c>
       <c r="M18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
@@ -2170,19 +2171,19 @@
         <v>103023</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E19">
         <v>3</v>
       </c>
       <c r="F19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I19">
         <v>1004</v>
@@ -2197,7 +2198,7 @@
         <v>100</v>
       </c>
       <c r="M19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
@@ -2205,22 +2206,22 @@
         <v>110001</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
@@ -2228,22 +2229,22 @@
         <v>110002</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E21">
         <v>2</v>
       </c>
       <c r="F21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
@@ -2251,22 +2252,22 @@
         <v>110003</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E22">
         <v>3</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
@@ -2274,22 +2275,22 @@
         <v>110004</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E23">
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
@@ -2297,22 +2298,22 @@
         <v>110005</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E24">
         <v>5</v>
       </c>
       <c r="F24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
@@ -2320,22 +2321,22 @@
         <v>111001</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
@@ -2343,22 +2344,22 @@
         <v>111002</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E26">
         <v>2</v>
       </c>
       <c r="F26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
@@ -2366,22 +2367,22 @@
         <v>111003</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E27">
         <v>3</v>
       </c>
       <c r="F27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
@@ -2389,22 +2390,22 @@
         <v>111004</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E28">
         <v>4</v>
       </c>
       <c r="F28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
@@ -2412,22 +2413,22 @@
         <v>111005</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" t="s">
         <v>70</v>
-      </c>
-      <c r="D29" t="s">
-        <v>71</v>
       </c>
       <c r="E29">
         <v>5</v>
       </c>
       <c r="F29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
@@ -2435,22 +2436,22 @@
         <v>112001</v>
       </c>
       <c r="B30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" t="s">
         <v>80</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>81</v>
-      </c>
-      <c r="D30" t="s">
-        <v>82</v>
       </c>
       <c r="E30">
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DrillData에 entity class 연결
+ 프리펩 연결 방식을 기존 Name에서 숫자 뗴던 방식에서 type으로 받아옴
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Coding\Drill_Game\Assets\100_Data\XlsxFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koseonghyeon\Desktop\Drill_Game\Drill_game\Assets\100_Data\XlsxFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1C4167-45DF-4D95-BC75-E4E23D49C7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Facility_Data" sheetId="1" r:id="rId1"/>
@@ -19,12 +20,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>HOME2</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -121,7 +122,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -195,7 +196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -302,7 +303,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="208">
   <si>
     <t>0,0</t>
   </si>
@@ -591,10 +592,6 @@
   </si>
   <si>
     <t>EntityClassName</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>FacilityEntity</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
@@ -1054,11 +1051,19 @@
     <t>resourceMergerIcon</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
+  <si>
+    <t>ResourceMergerEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>EngineMergerEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1735,38 +1740,32 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1828,26 +1827,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="표2" displayName="표2" ref="A1:Q67" totalsRowShown="0">
-  <autoFilter ref="A1:Q67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표2" displayName="표2" ref="A1:Q67" totalsRowShown="0">
+  <autoFilter ref="A1:Q67" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="Id"/>
-    <tableColumn id="5" name="Name"/>
-    <tableColumn id="2" name="DisplayName"/>
-    <tableColumn id="8" name="Type"/>
-    <tableColumn id="14" name="Icon"/>
-    <tableColumn id="3" name="Level"/>
-    <tableColumn id="13" name="EntityClassName"/>
-    <tableColumn id="15" name="Desc"/>
-    <tableColumn id="16" name="RequireResearchId"/>
-    <tableColumn id="18" name="RequireCoreLevel"/>
-    <tableColumn id="11" name="BuildResourceId"/>
-    <tableColumn id="12" name="BuildResourceCount"/>
-    <tableColumn id="7" name="InputItemId"/>
-    <tableColumn id="10" name="InputItemCount"/>
-    <tableColumn id="6" name="OutputItemId"/>
-    <tableColumn id="9" name="OutputItemCount"/>
-    <tableColumn id="4" name="Coordinates"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DisplayName"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Type"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Icon"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Level"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="EntityClassName"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Desc"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="RequireResearchId"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="RequireCoreLevel"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="BuildResourceId"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="BuildResourceCount"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="InputItemId"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="InputItemCount"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="OutputItemId"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="OutputItemCount"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Coordinates"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2115,7 +2114,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q67"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2146,7 +2145,7 @@
         <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
@@ -2158,10 +2157,10 @@
         <v>66</v>
       </c>
       <c r="I1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K1" t="s">
         <v>40</v>
@@ -2199,13 +2198,13 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H2" t="s">
         <v>71</v>
@@ -2213,7 +2212,7 @@
       <c r="K2">
         <v>1002</v>
       </c>
-      <c r="L2" s="10">
+      <c r="L2">
         <v>10000</v>
       </c>
       <c r="O2">
@@ -2240,13 +2239,13 @@
         <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H3" t="s">
         <v>72</v>
@@ -2254,7 +2253,7 @@
       <c r="K3">
         <v>1002</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3">
         <v>10000</v>
       </c>
       <c r="M3">
@@ -2287,13 +2286,13 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H4" t="s">
         <v>73</v>
@@ -2304,7 +2303,7 @@
       <c r="K4">
         <v>1002</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4">
         <v>200</v>
       </c>
       <c r="O4">
@@ -2331,13 +2330,13 @@
         <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F5">
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H5" t="s">
         <v>74</v>
@@ -2348,7 +2347,7 @@
       <c r="K5">
         <v>1004</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L5">
         <v>2000</v>
       </c>
       <c r="O5">
@@ -2358,7 +2357,7 @@
         <v>10</v>
       </c>
       <c r="Q5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -2375,13 +2374,13 @@
         <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F6">
         <v>3</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H6" t="s">
         <v>75</v>
@@ -2392,7 +2391,7 @@
       <c r="K6">
         <v>1004</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6">
         <v>30000</v>
       </c>
       <c r="O6">
@@ -2402,7 +2401,7 @@
         <v>100</v>
       </c>
       <c r="Q6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -2419,13 +2418,13 @@
         <v>14</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H7" t="s">
         <v>76</v>
@@ -2436,7 +2435,7 @@
       <c r="K7">
         <v>1002</v>
       </c>
-      <c r="L7" s="10">
+      <c r="L7">
         <v>200</v>
       </c>
       <c r="M7">
@@ -2469,13 +2468,13 @@
         <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H8" t="s">
         <v>76</v>
@@ -2486,7 +2485,7 @@
       <c r="K8">
         <v>1004</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8">
         <v>2000</v>
       </c>
       <c r="M8">
@@ -2502,7 +2501,7 @@
         <v>10</v>
       </c>
       <c r="Q8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -2519,13 +2518,13 @@
         <v>14</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H9" t="s">
         <v>77</v>
@@ -2536,7 +2535,7 @@
       <c r="K9">
         <v>1004</v>
       </c>
-      <c r="L9" s="10">
+      <c r="L9">
         <v>30000</v>
       </c>
       <c r="M9">
@@ -2552,7 +2551,7 @@
         <v>100</v>
       </c>
       <c r="Q9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -2569,13 +2568,13 @@
         <v>10</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H10" t="s">
         <v>69</v>
@@ -2586,7 +2585,7 @@
       <c r="K10">
         <v>1004</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10">
         <v>40000</v>
       </c>
       <c r="O10">
@@ -2613,13 +2612,13 @@
         <v>10</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H11" t="s">
         <v>69</v>
@@ -2630,7 +2629,7 @@
       <c r="K11">
         <v>1006</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11">
         <v>2000</v>
       </c>
       <c r="O11">
@@ -2640,7 +2639,7 @@
         <v>10</v>
       </c>
       <c r="Q11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -2657,13 +2656,13 @@
         <v>10</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F12">
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H12" t="s">
         <v>69</v>
@@ -2674,7 +2673,7 @@
       <c r="K12">
         <v>1006</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L12">
         <v>30000</v>
       </c>
       <c r="O12">
@@ -2684,7 +2683,7 @@
         <v>100</v>
       </c>
       <c r="Q12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -2701,13 +2700,13 @@
         <v>14</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H13" t="s">
         <v>70</v>
@@ -2718,7 +2717,7 @@
       <c r="K13">
         <v>1004</v>
       </c>
-      <c r="L13" s="10">
+      <c r="L13">
         <v>40000</v>
       </c>
       <c r="M13">
@@ -2751,13 +2750,13 @@
         <v>14</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H14" t="s">
         <v>70</v>
@@ -2768,7 +2767,7 @@
       <c r="K14">
         <v>1006</v>
       </c>
-      <c r="L14" s="10">
+      <c r="L14">
         <v>2000</v>
       </c>
       <c r="M14">
@@ -2784,7 +2783,7 @@
         <v>10</v>
       </c>
       <c r="Q14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -2801,13 +2800,13 @@
         <v>14</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
       <c r="G15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H15" t="s">
         <v>70</v>
@@ -2818,7 +2817,7 @@
       <c r="K15">
         <v>1006</v>
       </c>
-      <c r="L15" s="10">
+      <c r="L15">
         <v>30000</v>
       </c>
       <c r="M15">
@@ -2834,7 +2833,7 @@
         <v>100</v>
       </c>
       <c r="Q15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -2842,25 +2841,25 @@
         <v>104011</v>
       </c>
       <c r="B16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I16">
         <v>30011</v>
@@ -2868,7 +2867,7 @@
       <c r="K16">
         <v>1006</v>
       </c>
-      <c r="L16" s="10">
+      <c r="L16">
         <v>40000</v>
       </c>
       <c r="O16">
@@ -2886,25 +2885,25 @@
         <v>104012</v>
       </c>
       <c r="B17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F17">
         <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H17" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I17">
         <v>30012</v>
@@ -2912,7 +2911,7 @@
       <c r="K17">
         <v>1008</v>
       </c>
-      <c r="L17" s="10">
+      <c r="L17">
         <v>2000</v>
       </c>
       <c r="O17">
@@ -2922,7 +2921,7 @@
         <v>10</v>
       </c>
       <c r="Q17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
@@ -2930,25 +2929,25 @@
         <v>104013</v>
       </c>
       <c r="B18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F18">
         <v>3</v>
       </c>
       <c r="G18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I18">
         <v>30013</v>
@@ -2956,7 +2955,7 @@
       <c r="K18">
         <v>1008</v>
       </c>
-      <c r="L18" s="10">
+      <c r="L18">
         <v>30000</v>
       </c>
       <c r="O18">
@@ -2966,7 +2965,7 @@
         <v>100</v>
       </c>
       <c r="Q18" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
@@ -2974,25 +2973,25 @@
         <v>104021</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D19" t="s">
         <v>14</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="G19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I19">
         <v>30011</v>
@@ -3000,7 +2999,7 @@
       <c r="K19">
         <v>1006</v>
       </c>
-      <c r="L19" s="10">
+      <c r="L19">
         <v>40000</v>
       </c>
       <c r="M19">
@@ -3024,25 +3023,25 @@
         <v>104022</v>
       </c>
       <c r="B20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
         <v>14</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F20">
         <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H20" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I20">
         <v>30012</v>
@@ -3050,7 +3049,7 @@
       <c r="K20">
         <v>1008</v>
       </c>
-      <c r="L20" s="10">
+      <c r="L20">
         <v>2000</v>
       </c>
       <c r="M20">
@@ -3066,7 +3065,7 @@
         <v>10</v>
       </c>
       <c r="Q20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
@@ -3074,25 +3073,25 @@
         <v>104023</v>
       </c>
       <c r="B21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D21" t="s">
         <v>14</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F21">
         <v>3</v>
       </c>
       <c r="G21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I21">
         <v>30013</v>
@@ -3100,7 +3099,7 @@
       <c r="K21">
         <v>1008</v>
       </c>
-      <c r="L21" s="10">
+      <c r="L21">
         <v>30000</v>
       </c>
       <c r="M21">
@@ -3116,7 +3115,7 @@
         <v>100</v>
       </c>
       <c r="Q21" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -3124,25 +3123,25 @@
         <v>105011</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I22">
         <v>30016</v>
@@ -3150,7 +3149,7 @@
       <c r="K22">
         <v>1008</v>
       </c>
-      <c r="L22" s="10">
+      <c r="L22">
         <v>40000</v>
       </c>
       <c r="O22">
@@ -3168,25 +3167,25 @@
         <v>105012</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F23">
         <v>2</v>
       </c>
       <c r="G23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I23">
         <v>30017</v>
@@ -3194,7 +3193,7 @@
       <c r="K23">
         <v>1010</v>
       </c>
-      <c r="L23" s="10">
+      <c r="L23">
         <v>2000</v>
       </c>
       <c r="O23">
@@ -3204,7 +3203,7 @@
         <v>10</v>
       </c>
       <c r="Q23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
@@ -3212,25 +3211,25 @@
         <v>105013</v>
       </c>
       <c r="B24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F24">
         <v>3</v>
       </c>
       <c r="G24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I24">
         <v>30018</v>
@@ -3238,7 +3237,7 @@
       <c r="K24">
         <v>1010</v>
       </c>
-      <c r="L24" s="10">
+      <c r="L24">
         <v>30000</v>
       </c>
       <c r="O24">
@@ -3248,7 +3247,7 @@
         <v>100</v>
       </c>
       <c r="Q24" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
@@ -3256,25 +3255,25 @@
         <v>105021</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D25" t="s">
         <v>14</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I25">
         <v>30016</v>
@@ -3282,7 +3281,7 @@
       <c r="K25">
         <v>1008</v>
       </c>
-      <c r="L25" s="10">
+      <c r="L25">
         <v>40000</v>
       </c>
       <c r="M25">
@@ -3306,25 +3305,25 @@
         <v>105022</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D26" t="s">
         <v>14</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
       <c r="G26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I26">
         <v>30017</v>
@@ -3332,7 +3331,7 @@
       <c r="K26">
         <v>1010</v>
       </c>
-      <c r="L26" s="10">
+      <c r="L26">
         <v>2000</v>
       </c>
       <c r="M26">
@@ -3348,7 +3347,7 @@
         <v>10</v>
       </c>
       <c r="Q26" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
@@ -3356,25 +3355,25 @@
         <v>105023</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D27" t="s">
         <v>14</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F27">
         <v>3</v>
       </c>
       <c r="G27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H27" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I27">
         <v>30018</v>
@@ -3382,7 +3381,7 @@
       <c r="K27">
         <v>1010</v>
       </c>
-      <c r="L27" s="10">
+      <c r="L27">
         <v>30000</v>
       </c>
       <c r="M27">
@@ -3398,7 +3397,7 @@
         <v>100</v>
       </c>
       <c r="Q27" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
@@ -3406,25 +3405,25 @@
         <v>106011</v>
       </c>
       <c r="B28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I28">
         <v>30021</v>
@@ -3432,7 +3431,7 @@
       <c r="K28">
         <v>1010</v>
       </c>
-      <c r="L28" s="10">
+      <c r="L28">
         <v>40000</v>
       </c>
       <c r="O28">
@@ -3450,25 +3449,25 @@
         <v>106012</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F29">
         <v>2</v>
       </c>
       <c r="G29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I29">
         <v>30022</v>
@@ -3476,7 +3475,7 @@
       <c r="K29">
         <v>1012</v>
       </c>
-      <c r="L29" s="10">
+      <c r="L29">
         <v>2000</v>
       </c>
       <c r="O29">
@@ -3486,7 +3485,7 @@
         <v>10</v>
       </c>
       <c r="Q29" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
@@ -3494,25 +3493,25 @@
         <v>106013</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F30">
         <v>3</v>
       </c>
       <c r="G30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H30" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I30">
         <v>30023</v>
@@ -3520,7 +3519,7 @@
       <c r="K30">
         <v>1012</v>
       </c>
-      <c r="L30" s="10">
+      <c r="L30">
         <v>30000</v>
       </c>
       <c r="O30">
@@ -3530,7 +3529,7 @@
         <v>100</v>
       </c>
       <c r="Q30" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
@@ -3538,25 +3537,25 @@
         <v>106021</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D31" t="s">
         <v>14</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H31" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I31">
         <v>30021</v>
@@ -3564,7 +3563,7 @@
       <c r="K31">
         <v>1010</v>
       </c>
-      <c r="L31" s="10">
+      <c r="L31">
         <v>40000</v>
       </c>
       <c r="M31">
@@ -3588,25 +3587,25 @@
         <v>106022</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C32" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D32" t="s">
         <v>14</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H32" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I32">
         <v>30022</v>
@@ -3614,7 +3613,7 @@
       <c r="K32">
         <v>1012</v>
       </c>
-      <c r="L32" s="10">
+      <c r="L32">
         <v>2000</v>
       </c>
       <c r="M32">
@@ -3630,7 +3629,7 @@
         <v>10</v>
       </c>
       <c r="Q32" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
@@ -3638,25 +3637,25 @@
         <v>106023</v>
       </c>
       <c r="B33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C33" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D33" t="s">
         <v>14</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F33">
         <v>3</v>
       </c>
       <c r="G33" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H33" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I33">
         <v>30023</v>
@@ -3664,7 +3663,7 @@
       <c r="K33">
         <v>1012</v>
       </c>
-      <c r="L33" s="10">
+      <c r="L33">
         <v>30000</v>
       </c>
       <c r="M33">
@@ -3680,7 +3679,7 @@
         <v>100</v>
       </c>
       <c r="Q33" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
@@ -3688,25 +3687,25 @@
         <v>107011</v>
       </c>
       <c r="B34" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C34" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H34" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I34">
         <v>30026</v>
@@ -3714,7 +3713,7 @@
       <c r="K34">
         <v>1012</v>
       </c>
-      <c r="L34" s="10">
+      <c r="L34">
         <v>40000</v>
       </c>
       <c r="O34">
@@ -3732,25 +3731,25 @@
         <v>107012</v>
       </c>
       <c r="B35" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F35">
         <v>2</v>
       </c>
       <c r="G35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H35" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I35">
         <v>30027</v>
@@ -3758,7 +3757,7 @@
       <c r="K35">
         <v>1012</v>
       </c>
-      <c r="L35" s="10">
+      <c r="L35">
         <v>2000</v>
       </c>
       <c r="O35">
@@ -3768,7 +3767,7 @@
         <v>10</v>
       </c>
       <c r="Q35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
@@ -3776,25 +3775,25 @@
         <v>107013</v>
       </c>
       <c r="B36" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C36" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F36">
         <v>3</v>
       </c>
       <c r="G36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H36" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I36">
         <v>30028</v>
@@ -3802,7 +3801,7 @@
       <c r="K36">
         <v>1012</v>
       </c>
-      <c r="L36" s="10">
+      <c r="L36">
         <v>30000</v>
       </c>
       <c r="O36">
@@ -3812,7 +3811,7 @@
         <v>100</v>
       </c>
       <c r="Q36" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
@@ -3820,25 +3819,25 @@
         <v>107021</v>
       </c>
       <c r="B37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D37" t="s">
         <v>14</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37" t="s">
-        <v>82</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>153</v>
+        <v>81</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="I37">
         <v>30026</v>
@@ -3846,7 +3845,7 @@
       <c r="K37">
         <v>1012</v>
       </c>
-      <c r="L37" s="10">
+      <c r="L37">
         <v>40000</v>
       </c>
       <c r="M37">
@@ -3870,25 +3869,25 @@
         <v>107022</v>
       </c>
       <c r="B38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D38" t="s">
         <v>14</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F38">
         <v>2</v>
       </c>
       <c r="G38" t="s">
-        <v>82</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>153</v>
+        <v>81</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="I38">
         <v>30027</v>
@@ -3896,7 +3895,7 @@
       <c r="K38">
         <v>1012</v>
       </c>
-      <c r="L38" s="10">
+      <c r="L38">
         <v>2000</v>
       </c>
       <c r="M38">
@@ -3912,7 +3911,7 @@
         <v>10</v>
       </c>
       <c r="Q38" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
@@ -3920,25 +3919,25 @@
         <v>107023</v>
       </c>
       <c r="B39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C39" t="s">
-        <v>150</v>
-      </c>
-      <c r="D39" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D39" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="F39" s="7">
+      <c r="E39" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39">
         <v>3</v>
       </c>
-      <c r="G39" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>153</v>
+      <c r="G39" t="s">
+        <v>81</v>
+      </c>
+      <c r="H39" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="I39">
         <v>30028</v>
@@ -3946,23 +3945,23 @@
       <c r="K39">
         <v>1012</v>
       </c>
-      <c r="L39" s="10">
+      <c r="L39">
         <v>30000</v>
       </c>
       <c r="M39">
         <v>1013</v>
       </c>
-      <c r="N39" s="7">
+      <c r="N39">
         <v>100</v>
       </c>
       <c r="O39">
         <v>1014</v>
       </c>
-      <c r="P39" s="7">
+      <c r="P39">
         <v>100</v>
       </c>
       <c r="Q39" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
@@ -3979,13 +3978,13 @@
         <v>59</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F40" s="4">
         <v>1</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>67</v>
@@ -3995,7 +3994,7 @@
       <c r="K40" s="4">
         <v>1002</v>
       </c>
-      <c r="L40" s="10">
+      <c r="L40">
         <v>5000</v>
       </c>
       <c r="M40" s="4"/>
@@ -4020,13 +4019,13 @@
         <v>59</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F41" s="6">
         <v>2</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>67</v>
@@ -4038,7 +4037,7 @@
       <c r="K41" s="6">
         <v>1004</v>
       </c>
-      <c r="L41" s="10">
+      <c r="L41">
         <v>20000</v>
       </c>
       <c r="M41" s="6"/>
@@ -4063,13 +4062,13 @@
         <v>59</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F42" s="6">
         <v>3</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>67</v>
@@ -4081,7 +4080,7 @@
       <c r="K42" s="4">
         <v>1006</v>
       </c>
-      <c r="L42" s="10">
+      <c r="L42">
         <v>20000</v>
       </c>
       <c r="M42" s="6"/>
@@ -4106,13 +4105,13 @@
         <v>59</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F43" s="6">
         <v>4</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>67</v>
@@ -4124,7 +4123,7 @@
       <c r="K43" s="6">
         <v>1008</v>
       </c>
-      <c r="L43" s="10">
+      <c r="L43">
         <v>20000</v>
       </c>
       <c r="M43" s="6"/>
@@ -4143,19 +4142,19 @@
         <v>64</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>59</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F44" s="6">
         <v>5</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>67</v>
@@ -4167,7 +4166,7 @@
       <c r="K44" s="4">
         <v>1010</v>
       </c>
-      <c r="L44" s="10">
+      <c r="L44">
         <v>20000</v>
       </c>
       <c r="M44" s="6"/>
@@ -4183,22 +4182,22 @@
         <v>110006</v>
       </c>
       <c r="B45" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C45" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>59</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F45" s="6">
         <v>6</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>67</v>
@@ -4210,7 +4209,7 @@
       <c r="K45" s="6">
         <v>1012</v>
       </c>
-      <c r="L45" s="10">
+      <c r="L45">
         <v>20000</v>
       </c>
       <c r="M45" s="6"/>
@@ -4226,22 +4225,22 @@
         <v>110007</v>
       </c>
       <c r="B46" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>189</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>190</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>59</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F46" s="6">
         <v>7</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>67</v>
@@ -4253,7 +4252,7 @@
       <c r="K46" s="4">
         <v>1014</v>
       </c>
-      <c r="L46" s="10">
+      <c r="L46">
         <v>20000</v>
       </c>
       <c r="M46" s="6"/>
@@ -4278,13 +4277,13 @@
         <v>58</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F47" s="6">
         <v>1</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>79</v>
+        <v>207</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>68</v>
@@ -4294,7 +4293,7 @@
       <c r="K47" s="6">
         <v>1002</v>
       </c>
-      <c r="L47" s="10">
+      <c r="L47">
         <v>5000</v>
       </c>
       <c r="M47" s="6"/>
@@ -4319,13 +4318,13 @@
         <v>58</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F48" s="4">
         <v>2</v>
       </c>
-      <c r="G48" s="4" t="s">
-        <v>79</v>
+      <c r="G48" s="6" t="s">
+        <v>207</v>
       </c>
       <c r="H48" s="4" t="s">
         <v>68</v>
@@ -4337,7 +4336,7 @@
       <c r="K48" s="4">
         <v>1004</v>
       </c>
-      <c r="L48" s="10">
+      <c r="L48">
         <v>20000</v>
       </c>
       <c r="M48" s="4"/>
@@ -4362,13 +4361,13 @@
         <v>58</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F49" s="6">
         <v>3</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>79</v>
+        <v>207</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>68</v>
@@ -4380,7 +4379,7 @@
       <c r="K49" s="6">
         <v>1006</v>
       </c>
-      <c r="L49" s="10">
+      <c r="L49">
         <v>20000</v>
       </c>
       <c r="M49" s="6"/>
@@ -4405,13 +4404,13 @@
         <v>58</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F50" s="4">
         <v>4</v>
       </c>
-      <c r="G50" s="4" t="s">
-        <v>79</v>
+      <c r="G50" s="6" t="s">
+        <v>207</v>
       </c>
       <c r="H50" s="4" t="s">
         <v>68</v>
@@ -4423,7 +4422,7 @@
       <c r="K50" s="4">
         <v>1008</v>
       </c>
-      <c r="L50" s="10">
+      <c r="L50">
         <v>20000</v>
       </c>
       <c r="M50" s="4"/>
@@ -4448,13 +4447,13 @@
         <v>58</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F51" s="6">
         <v>5</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>79</v>
+        <v>207</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>68</v>
@@ -4466,7 +4465,7 @@
       <c r="K51" s="6">
         <v>1010</v>
       </c>
-      <c r="L51" s="10">
+      <c r="L51">
         <v>20000</v>
       </c>
       <c r="M51" s="6"/>
@@ -4482,22 +4481,22 @@
         <v>111006</v>
       </c>
       <c r="B52" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" s="6" t="s">
         <v>174</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>175</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F52" s="6">
         <v>6</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>79</v>
+        <v>207</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>68</v>
@@ -4509,7 +4508,7 @@
       <c r="K52" s="6">
         <v>1012</v>
       </c>
-      <c r="L52" s="10">
+      <c r="L52">
         <v>20000</v>
       </c>
       <c r="M52" s="6"/>
@@ -4525,22 +4524,22 @@
         <v>111007</v>
       </c>
       <c r="B53" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C53" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>177</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F53" s="6">
         <v>7</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>79</v>
+        <v>207</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>68</v>
@@ -4552,7 +4551,7 @@
       <c r="K53" s="6">
         <v>1014</v>
       </c>
-      <c r="L53" s="10">
+      <c r="L53">
         <v>20000</v>
       </c>
       <c r="M53" s="6"/>
@@ -4564,39 +4563,31 @@
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A54" s="10">
+      <c r="A54">
         <v>112001</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="B54" t="s">
+        <v>177</v>
+      </c>
+      <c r="C54" t="s">
+        <v>167</v>
+      </c>
+      <c r="D54" t="s">
         <v>178</v>
       </c>
-      <c r="C54" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="D54" s="10" t="s">
+      <c r="E54" t="s">
         <v>179</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="F54">
+        <v>1</v>
+      </c>
+      <c r="G54" t="s">
         <v>180</v>
       </c>
-      <c r="F54" s="10">
-        <v>1</v>
-      </c>
-      <c r="G54" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="H54" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="I54" s="10"/>
-      <c r="J54" s="10"/>
-      <c r="K54" s="10"/>
-      <c r="L54" s="10"/>
-      <c r="M54" s="10"/>
-      <c r="N54" s="10"/>
-      <c r="O54" s="10"/>
-      <c r="P54" s="10"/>
-      <c r="Q54" s="10" t="s">
+      <c r="H54" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q54" t="s">
         <v>0</v>
       </c>
     </row>
@@ -4605,25 +4596,25 @@
         <v>112002</v>
       </c>
       <c r="B55" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D55" t="s">
+        <v>178</v>
+      </c>
+      <c r="E55" t="s">
         <v>179</v>
-      </c>
-      <c r="E55" t="s">
-        <v>180</v>
       </c>
       <c r="F55">
         <v>2</v>
       </c>
       <c r="G55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I55">
         <v>30005</v>
@@ -4637,25 +4628,25 @@
         <v>112003</v>
       </c>
       <c r="B56" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C56" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D56" t="s">
+        <v>178</v>
+      </c>
+      <c r="E56" t="s">
         <v>179</v>
-      </c>
-      <c r="E56" t="s">
-        <v>180</v>
       </c>
       <c r="F56">
         <v>3</v>
       </c>
       <c r="G56" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H56" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I56">
         <v>30010</v>
@@ -4669,25 +4660,25 @@
         <v>112004</v>
       </c>
       <c r="B57" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C57" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D57" t="s">
+        <v>178</v>
+      </c>
+      <c r="E57" t="s">
         <v>179</v>
-      </c>
-      <c r="E57" t="s">
-        <v>180</v>
       </c>
       <c r="F57">
         <v>4</v>
       </c>
       <c r="G57" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H57" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I57">
         <v>30015</v>
@@ -4701,25 +4692,25 @@
         <v>112005</v>
       </c>
       <c r="B58" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C58" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D58" t="s">
+        <v>178</v>
+      </c>
+      <c r="E58" t="s">
         <v>179</v>
-      </c>
-      <c r="E58" t="s">
-        <v>180</v>
       </c>
       <c r="F58">
         <v>5</v>
       </c>
       <c r="G58" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H58" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I58">
         <v>30020</v>
@@ -4733,25 +4724,25 @@
         <v>112006</v>
       </c>
       <c r="B59" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C59" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D59" t="s">
+        <v>178</v>
+      </c>
+      <c r="E59" t="s">
         <v>179</v>
-      </c>
-      <c r="E59" t="s">
-        <v>180</v>
       </c>
       <c r="F59">
         <v>6</v>
       </c>
       <c r="G59" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H59" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I59">
         <v>30025</v>
@@ -4765,25 +4756,25 @@
         <v>112007</v>
       </c>
       <c r="B60" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C60" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D60" t="s">
+        <v>178</v>
+      </c>
+      <c r="E60" t="s">
         <v>179</v>
-      </c>
-      <c r="E60" t="s">
-        <v>180</v>
       </c>
       <c r="F60">
         <v>7</v>
       </c>
       <c r="G60" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H60" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I60">
         <v>30030</v>
@@ -4797,34 +4788,34 @@
         <v>113001</v>
       </c>
       <c r="B61" t="s">
+        <v>181</v>
+      </c>
+      <c r="C61" t="s">
         <v>182</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
         <v>183</v>
       </c>
-      <c r="D61" t="s">
-        <v>184</v>
-      </c>
       <c r="E61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F61">
         <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H61" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K61">
         <v>1002</v>
       </c>
-      <c r="L61" s="10">
+      <c r="L61">
         <v>5000</v>
       </c>
       <c r="Q61" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.3">
@@ -4832,25 +4823,25 @@
         <v>113002</v>
       </c>
       <c r="B62" t="s">
+        <v>191</v>
+      </c>
+      <c r="C62" t="s">
         <v>192</v>
       </c>
-      <c r="C62" t="s">
-        <v>193</v>
-      </c>
       <c r="D62" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E62" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F62">
         <v>2</v>
       </c>
       <c r="G62" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H62" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J62" s="6">
         <v>2</v>
@@ -4858,11 +4849,11 @@
       <c r="K62">
         <v>1004</v>
       </c>
-      <c r="L62" s="10">
+      <c r="L62">
         <v>20000</v>
       </c>
       <c r="Q62" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.3">
@@ -4870,25 +4861,25 @@
         <v>113003</v>
       </c>
       <c r="B63" t="s">
+        <v>193</v>
+      </c>
+      <c r="C63" t="s">
         <v>194</v>
       </c>
-      <c r="C63" t="s">
-        <v>195</v>
-      </c>
       <c r="D63" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E63" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F63">
         <v>3</v>
       </c>
       <c r="G63" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H63" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J63" s="6">
         <v>3</v>
@@ -4896,11 +4887,11 @@
       <c r="K63">
         <v>1006</v>
       </c>
-      <c r="L63" s="10">
+      <c r="L63">
         <v>20000</v>
       </c>
       <c r="Q63" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.3">
@@ -4908,25 +4899,25 @@
         <v>113004</v>
       </c>
       <c r="B64" t="s">
+        <v>195</v>
+      </c>
+      <c r="C64" t="s">
         <v>196</v>
       </c>
-      <c r="C64" t="s">
-        <v>197</v>
-      </c>
       <c r="D64" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E64" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F64">
         <v>4</v>
       </c>
       <c r="G64" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H64" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J64" s="6">
         <v>4</v>
@@ -4934,11 +4925,11 @@
       <c r="K64">
         <v>1008</v>
       </c>
-      <c r="L64" s="10">
+      <c r="L64">
         <v>20000</v>
       </c>
       <c r="Q64" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.3">
@@ -4946,25 +4937,25 @@
         <v>113005</v>
       </c>
       <c r="B65" t="s">
+        <v>197</v>
+      </c>
+      <c r="C65" t="s">
         <v>198</v>
       </c>
-      <c r="C65" t="s">
-        <v>199</v>
-      </c>
       <c r="D65" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E65" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F65">
         <v>5</v>
       </c>
       <c r="G65" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H65" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J65" s="6">
         <v>5</v>
@@ -4972,11 +4963,11 @@
       <c r="K65">
         <v>1010</v>
       </c>
-      <c r="L65" s="10">
+      <c r="L65">
         <v>20000</v>
       </c>
       <c r="Q65" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.3">
@@ -4984,25 +4975,25 @@
         <v>113006</v>
       </c>
       <c r="B66" t="s">
+        <v>199</v>
+      </c>
+      <c r="C66" t="s">
         <v>200</v>
       </c>
-      <c r="C66" t="s">
-        <v>201</v>
-      </c>
       <c r="D66" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E66" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F66">
         <v>6</v>
       </c>
       <c r="G66" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H66" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J66" s="6">
         <v>6</v>
@@ -5010,11 +5001,11 @@
       <c r="K66">
         <v>1012</v>
       </c>
-      <c r="L66" s="10">
+      <c r="L66">
         <v>20000</v>
       </c>
       <c r="Q66" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.3">
@@ -5022,25 +5013,25 @@
         <v>113007</v>
       </c>
       <c r="B67" t="s">
+        <v>201</v>
+      </c>
+      <c r="C67" t="s">
         <v>202</v>
       </c>
-      <c r="C67" t="s">
-        <v>203</v>
-      </c>
       <c r="D67" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E67" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F67">
         <v>7</v>
       </c>
       <c r="G67" t="s">
-        <v>79</v>
+        <v>206</v>
       </c>
       <c r="H67" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J67" s="6">
         <v>7</v>
@@ -5048,7 +5039,7 @@
       <c r="K67">
         <v>1014</v>
       </c>
-      <c r="L67" s="10">
+      <c r="L67">
         <v>20000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Facility Sprite들 Addressable 지정
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Facility_Data.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koseonghyeon\Desktop\Drill_Game\Drill_game\Assets\100_Data\XlsxFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Coding\Drill_Game\Assets\100_Data\XlsxFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{468F5478-78DB-4502-B145-A771C363A6F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Facility_Data" sheetId="1" r:id="rId1"/>
@@ -20,12 +19,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>HOME2</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -122,7 +121,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -196,7 +195,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -303,7 +302,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="199">
   <si>
     <t>0,0</t>
   </si>
@@ -475,614 +474,538 @@
     <t>연구소 Lv.4</t>
   </si>
   <si>
+    <t>stone_processor1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_merger1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_merger3</t>
+  </si>
+  <si>
+    <t>engine_merger4</t>
+  </si>
+  <si>
+    <t>engine_merger5</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.2</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.3</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.4</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.5</t>
+  </si>
+  <si>
+    <t>EngineMerger</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Laboratory</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>laboratory1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>laboratory2</t>
+  </si>
+  <si>
+    <t>laboratory3</t>
+  </si>
+  <si>
+    <t>laboratory4</t>
+  </si>
+  <si>
+    <t>laboratory5</t>
+  </si>
+  <si>
+    <t>Coordinates</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Desc</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>연구를 진행하여 공장을 강화할 수 있다.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>새로운 엔진을 개발하거나, 기존의 엔진들을 합성할 수 있다.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>EntityClassName</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>MinerEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>LabEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>ProcessEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Icon</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>RequireResearchId</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>금 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>금 채굴 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>금 채굴 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>gold_miner1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_processor1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>금 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>금 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>obsidian_miner1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_miner2</t>
+  </si>
+  <si>
+    <t>obsidian_miner3</t>
+  </si>
+  <si>
+    <t>obsidian_processor1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_processor2</t>
+  </si>
+  <si>
+    <t>obsidian_processor3</t>
+  </si>
+  <si>
+    <t>금 가공 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 채굴 시설 Lv.2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 채굴 시설 Lv.3</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 가공 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>흑요석 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>tunstein_miner1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_miner2</t>
+  </si>
+  <si>
+    <t>gold_miner3</t>
+  </si>
+  <si>
+    <t>gold_processor2</t>
+  </si>
+  <si>
+    <t>gold_processor3</t>
+  </si>
+  <si>
+    <t>tunstein_miner2</t>
+  </si>
+  <si>
+    <t>tunstein_miner3</t>
+  </si>
+  <si>
+    <t>tunstein_processor1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>tunstein_processor2</t>
+  </si>
+  <si>
+    <t>tunstein_processor3</t>
+  </si>
+  <si>
+    <t>텅스텐 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>텅스텐 채굴 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>텅스텐 채굴 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>텅스텐 가공 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>텅스텐 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>텅스텐 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>titanium_miner1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_miner2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_miner3</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_processor1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_processor2</t>
+  </si>
+  <si>
+    <t>titanium_processor3</t>
+  </si>
+  <si>
+    <t>티타늄 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 채굴 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>티타늄 가공 시설 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>티타늄 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>티타늄 채굴 시설 Lv.3</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>구리 드릴</t>
+  </si>
+  <si>
+    <t>거대 구리 드릴을 작동하기 위한 모터 시설이다.</t>
+  </si>
+  <si>
+    <t>drill2</t>
+  </si>
+  <si>
+    <t>drill3</t>
+  </si>
+  <si>
+    <t>drill4</t>
+  </si>
+  <si>
+    <t>drill5</t>
+  </si>
+  <si>
+    <t>drill6</t>
+  </si>
+  <si>
+    <t>drill7</t>
+  </si>
+  <si>
+    <t>거대 돌 드릴을 작동하기 위한 모터 시설이다.</t>
+  </si>
+  <si>
+    <t>거대 철 드릴을 작동하기 위한 모터 시설이다.</t>
+  </si>
+  <si>
+    <t>거대 금 드릴을 작동하기 위한 모터 시설이다.</t>
+  </si>
+  <si>
+    <t>거대 흑요석 드릴을 작동하기 위한 모터 시설이다.</t>
+  </si>
+  <si>
+    <t>거대 텅스텐 드릴을 작동하기 위한 모터 시설이다.</t>
+  </si>
+  <si>
+    <t>돌 드릴</t>
+  </si>
+  <si>
+    <t>철 드릴</t>
+  </si>
+  <si>
+    <t>금 드릴</t>
+  </si>
+  <si>
+    <t>흑요석 드릴</t>
+  </si>
+  <si>
+    <t>텅스텐 드릴</t>
+  </si>
+  <si>
+    <t>티타늄 드릴</t>
+  </si>
+  <si>
+    <t>engine_merger6</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.6</t>
+  </si>
+  <si>
+    <t>engine_merger7</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.7</t>
+  </si>
+  <si>
+    <t>drill1</t>
+  </si>
+  <si>
+    <t>Drill</t>
+  </si>
+  <si>
+    <t>DrillEntity</t>
+  </si>
+  <si>
+    <t>resource_merger1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>잉여 자원을 재활용하기 위한 시설이다.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>RequireCoreLevel</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>laboratory6</t>
+  </si>
+  <si>
+    <t>연구소 Lv.6</t>
+  </si>
+  <si>
+    <t>laboratory7</t>
+  </si>
+  <si>
+    <t>연구소 Lv.7</t>
+  </si>
+  <si>
+    <t>연구소 Lv.5</t>
+  </si>
+  <si>
+    <t>resource_merger2</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.2</t>
+  </si>
+  <si>
+    <t>resource_merger3</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.3</t>
+  </si>
+  <si>
+    <t>resource_merger4</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.4</t>
+  </si>
+  <si>
+    <t>resource_merger5</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.5</t>
+  </si>
+  <si>
+    <t>resource_merger6</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.6</t>
+  </si>
+  <si>
+    <t>resource_merger7</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.7</t>
+  </si>
+  <si>
+    <t>EngineMergerEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_merger2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>거대 티타늄 드릴을 작동하기 위한 모터 시설이다.</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Length</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>1,1</t>
+  </si>
+  <si>
+    <t>1,1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>2,2</t>
+  </si>
+  <si>
+    <t>2,2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>ResourceConverterEntity</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>ResourceConverter</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0;0,1;1,0;1,1</t>
+  </si>
+  <si>
     <t>stone_miner1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>stone_processor1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_merger1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_merger3</t>
-  </si>
-  <si>
-    <t>engine_merger4</t>
-  </si>
-  <si>
-    <t>engine_merger5</t>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.2</t>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.3</t>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.4</t>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.5</t>
-  </si>
-  <si>
-    <t>EngineMerger</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Laboratory</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>laboratory1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>laboratory2</t>
-  </si>
-  <si>
-    <t>laboratory3</t>
-  </si>
-  <si>
-    <t>laboratory4</t>
-  </si>
-  <si>
-    <t>laboratory5</t>
-  </si>
-  <si>
-    <t>Coordinates</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Desc</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>연구를 진행하여 공장을 강화할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>새로운 엔진을 개발하거나, 기존의 엔진들을 합성할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>철 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>철 광석을 철 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>돌 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>돌 광석을 돌 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>구리 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>구리 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>구리 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>구리 광석을 구리 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>구리 광석을 구리 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>EntityClassName</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>MinerEntity</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>LabEntity</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>ProcessEntity</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Icon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_test</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_test</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_test</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_test</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_test</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_test</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>labIcon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>labIcon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engineMergerIcon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engineMergerIcon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engineMergerIcon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>RequireResearchId</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>금 채굴 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>금 채굴 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>금 채굴 시설 Lv.3</t>
-  </si>
-  <si>
-    <t>gold_miner1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>gold_processor1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>금 가공 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>금 가공 시설 Lv.3</t>
-  </si>
-  <si>
-    <t>obsidian_miner1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>obsidian_miner2</t>
-  </si>
-  <si>
-    <t>obsidian_miner3</t>
-  </si>
-  <si>
-    <t>obsidian_processor1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>obsidian_processor2</t>
-  </si>
-  <si>
-    <t>obsidian_processor3</t>
-  </si>
-  <si>
-    <t>금 가공 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 채굴 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 채굴 시설 Lv.2</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 채굴 시설 Lv.3</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 가공 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 가공 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>흑요석 가공 시설 Lv.3</t>
-  </si>
-  <si>
-    <t>금 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>금 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>금 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>tunstein_miner1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>gold_miner2</t>
-  </si>
-  <si>
-    <t>gold_miner3</t>
-  </si>
-  <si>
-    <t>gold_processor2</t>
-  </si>
-  <si>
-    <t>gold_processor3</t>
-  </si>
-  <si>
-    <t>tunstein_miner2</t>
-  </si>
-  <si>
-    <t>tunstein_miner3</t>
-  </si>
-  <si>
-    <t>tunstein_processor1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>tunstein_processor2</t>
-  </si>
-  <si>
-    <t>tunstein_processor3</t>
-  </si>
-  <si>
-    <t>텅스텐 채굴 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>텅스텐 채굴 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>텅스텐 채굴 시설 Lv.3</t>
-  </si>
-  <si>
-    <t>텅스텐 가공 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>텅스텐 가공 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>텅스텐 가공 시설 Lv.3</t>
-  </si>
-  <si>
-    <t>텅스텐 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>텅스텐 광석을 텅스텐 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>흑요석 광석을 흑요석 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>금 광석을 금 자재로 가공할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>titanium_miner1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>titanium_miner2</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>titanium_miner3</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>titanium_processor1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>titanium_processor2</t>
-  </si>
-  <si>
-    <t>titanium_processor3</t>
-  </si>
-  <si>
-    <t>티타늄 채굴 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>티타늄 채굴 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>티타늄 가공 시설 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>티타늄 가공 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>티타늄 가공 시설 Lv.3</t>
-  </si>
-  <si>
-    <t>티타늄 채굴 시설 Lv.3</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>티타늄 광석을 생산할 수 있다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>티타늄</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 광석을 티타늄 자재로 가공할 수 있다.</t>
-    </r>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>구리 드릴</t>
-  </si>
-  <si>
-    <t>거대 구리 드릴을 작동하기 위한 모터 시설이다.</t>
-  </si>
-  <si>
-    <t>drill2</t>
-  </si>
-  <si>
-    <t>drill3</t>
-  </si>
-  <si>
-    <t>drill4</t>
-  </si>
-  <si>
-    <t>drill5</t>
-  </si>
-  <si>
-    <t>drill6</t>
-  </si>
-  <si>
-    <t>drill7</t>
-  </si>
-  <si>
-    <t>거대 돌 드릴을 작동하기 위한 모터 시설이다.</t>
-  </si>
-  <si>
-    <t>거대 철 드릴을 작동하기 위한 모터 시설이다.</t>
-  </si>
-  <si>
-    <t>거대 금 드릴을 작동하기 위한 모터 시설이다.</t>
-  </si>
-  <si>
-    <t>거대 흑요석 드릴을 작동하기 위한 모터 시설이다.</t>
-  </si>
-  <si>
-    <t>거대 텅스텐 드릴을 작동하기 위한 모터 시설이다.</t>
-  </si>
-  <si>
-    <t>돌 드릴</t>
-  </si>
-  <si>
-    <t>철 드릴</t>
-  </si>
-  <si>
-    <t>금 드릴</t>
-  </si>
-  <si>
-    <t>흑요석 드릴</t>
-  </si>
-  <si>
-    <t>텅스텐 드릴</t>
-  </si>
-  <si>
-    <t>티타늄 드릴</t>
-  </si>
-  <si>
-    <t>engine_merger6</t>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.6</t>
-  </si>
-  <si>
-    <t>engine_merger7</t>
-  </si>
-  <si>
-    <t>엔진 합성기 Lv.7</t>
-  </si>
-  <si>
-    <t>drill1</t>
-  </si>
-  <si>
-    <t>Drill</t>
-  </si>
-  <si>
-    <t>drillIcon</t>
-  </si>
-  <si>
-    <t>DrillEntity</t>
-  </si>
-  <si>
-    <t>resource_merger1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>잉여 자원을 재활용하기 위한 시설이다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>RequireCoreLevel</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>laboratory6</t>
-  </si>
-  <si>
-    <t>연구소 Lv.6</t>
-  </si>
-  <si>
-    <t>laboratory7</t>
-  </si>
-  <si>
-    <t>연구소 Lv.7</t>
-  </si>
-  <si>
-    <t>연구소 Lv.5</t>
-  </si>
-  <si>
-    <t>resource_merger2</t>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.2</t>
-  </si>
-  <si>
-    <t>resource_merger3</t>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.3</t>
-  </si>
-  <si>
-    <t>resource_merger4</t>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.4</t>
-  </si>
-  <si>
-    <t>resource_merger5</t>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.5</t>
-  </si>
-  <si>
-    <t>resource_merger6</t>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.6</t>
-  </si>
-  <si>
-    <t>resource_merger7</t>
-  </si>
-  <si>
-    <t>자원 합성기 Lv.7</t>
-  </si>
-  <si>
-    <t>EngineMergerEntity</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>engine_merger2</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>거대 티타늄 드릴을 작동하기 위한 모터 시설이다.</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>Length</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>1,1</t>
-  </si>
-  <si>
-    <t>1,1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>2,2</t>
-  </si>
-  <si>
-    <t>2,2</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>ResourceConverterEntity</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>resourceConverterIcon</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>ResourceConverter</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>0,0</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>0,0;0,1;1,0;1,1</t>
+    <t>stone_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>stone_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>copper_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>copper_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>iron_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>iron_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>tunstein_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>tunstein_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_miner</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_processor</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>laboratory</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>engine_merger</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>drill</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>resource_merger</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1467,7 +1390,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1619,17 +1542,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1759,7 +1671,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1779,9 +1691,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -1846,27 +1755,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표2" displayName="표2" ref="A1:R67" totalsRowShown="0">
-  <autoFilter ref="A1:R67" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="표2" displayName="표2" ref="A1:R67" totalsRowShown="0">
+  <autoFilter ref="A1:R67"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DisplayName"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Type"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Icon"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Level"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="EntityClassName"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Desc"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="RequireResearchId"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="RequireCoreLevel"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="BuildResourceId"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="BuildResourceCount"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="InputItemId"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="InputItemCount"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="OutputItemId"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="OutputItemCount"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Coordinates"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Length"/>
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="5" name="Name"/>
+    <tableColumn id="2" name="DisplayName"/>
+    <tableColumn id="8" name="Type"/>
+    <tableColumn id="14" name="Icon"/>
+    <tableColumn id="3" name="Level"/>
+    <tableColumn id="13" name="EntityClassName"/>
+    <tableColumn id="15" name="Desc"/>
+    <tableColumn id="16" name="RequireResearchId"/>
+    <tableColumn id="18" name="RequireCoreLevel"/>
+    <tableColumn id="11" name="BuildResourceId"/>
+    <tableColumn id="12" name="BuildResourceCount"/>
+    <tableColumn id="7" name="InputItemId"/>
+    <tableColumn id="10" name="InputItemCount"/>
+    <tableColumn id="6" name="OutputItemId"/>
+    <tableColumn id="9" name="OutputItemCount"/>
+    <tableColumn id="4" name="Coordinates"/>
+    <tableColumn id="17" name="Length"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2134,7 +2043,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R67"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2167,22 +2076,22 @@
         <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="H1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I1" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="J1" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="K1" t="s">
         <v>40</v>
@@ -2203,10 +2112,10 @@
         <v>16</v>
       </c>
       <c r="Q1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="R1" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -2214,7 +2123,7 @@
         <v>101011</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>180</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -2222,17 +2131,14 @@
       <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>82</v>
+      <c r="E2" t="s">
+        <v>181</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K2">
         <v>1002</v>
@@ -2250,7 +2156,7 @@
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -2258,7 +2164,7 @@
         <v>101021</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -2266,17 +2172,14 @@
       <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>83</v>
+      <c r="E3" t="s">
+        <v>182</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>80</v>
-      </c>
-      <c r="H3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K3">
         <v>1002</v>
@@ -2300,7 +2203,7 @@
         <v>0</v>
       </c>
       <c r="R3" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
@@ -2316,17 +2219,14 @@
       <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>84</v>
+      <c r="E4" t="s">
+        <v>183</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I4">
         <v>30001</v>
@@ -2347,7 +2247,7 @@
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
@@ -2363,17 +2263,14 @@
       <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>82</v>
+      <c r="E5" t="s">
+        <v>183</v>
       </c>
       <c r="F5">
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I5">
         <v>30002</v>
@@ -2391,10 +2288,10 @@
         <v>10</v>
       </c>
       <c r="Q5" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="R5" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
@@ -2410,17 +2307,14 @@
       <c r="D6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>85</v>
+      <c r="E6" t="s">
+        <v>183</v>
       </c>
       <c r="F6">
         <v>3</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I6">
         <v>30003</v>
@@ -2438,10 +2332,10 @@
         <v>100</v>
       </c>
       <c r="Q6" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="R6" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
@@ -2457,17 +2351,14 @@
       <c r="D7" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>86</v>
+      <c r="E7" t="s">
+        <v>184</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>80</v>
-      </c>
-      <c r="H7" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I7">
         <v>30001</v>
@@ -2494,7 +2385,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
@@ -2510,17 +2401,14 @@
       <c r="D8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>84</v>
+      <c r="E8" t="s">
+        <v>184</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>80</v>
-      </c>
-      <c r="H8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I8">
         <v>30002</v>
@@ -2544,10 +2432,10 @@
         <v>10</v>
       </c>
       <c r="Q8" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="R8" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
@@ -2563,17 +2451,14 @@
       <c r="D9" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>86</v>
+      <c r="E9" t="s">
+        <v>184</v>
       </c>
       <c r="F9">
         <v>3</v>
       </c>
       <c r="G9" t="s">
-        <v>80</v>
-      </c>
-      <c r="H9" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I9">
         <v>30003</v>
@@ -2597,10 +2482,10 @@
         <v>100</v>
       </c>
       <c r="Q9" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="R9" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
@@ -2616,16 +2501,13 @@
       <c r="D10" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>87</v>
+      <c r="E10" t="s">
+        <v>185</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H10" t="s">
         <v>68</v>
       </c>
       <c r="I10">
@@ -2647,7 +2529,7 @@
         <v>0</v>
       </c>
       <c r="R10" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -2663,16 +2545,13 @@
       <c r="D11" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>87</v>
+      <c r="E11" t="s">
+        <v>185</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" t="s">
         <v>68</v>
       </c>
       <c r="I11">
@@ -2691,10 +2570,10 @@
         <v>10</v>
       </c>
       <c r="Q11" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="R11" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
@@ -2710,16 +2589,13 @@
       <c r="D12" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>87</v>
+      <c r="E12" t="s">
+        <v>185</v>
       </c>
       <c r="F12">
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
-      </c>
-      <c r="H12" t="s">
         <v>68</v>
       </c>
       <c r="I12">
@@ -2741,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="R12" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
@@ -2757,17 +2633,14 @@
       <c r="D13" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>87</v>
+      <c r="E13" t="s">
+        <v>186</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>80</v>
-      </c>
-      <c r="H13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I13">
         <v>30006</v>
@@ -2794,7 +2667,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
@@ -2810,17 +2683,14 @@
       <c r="D14" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>87</v>
+      <c r="E14" t="s">
+        <v>186</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
-      </c>
-      <c r="H14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I14">
         <v>30007</v>
@@ -2847,7 +2717,7 @@
         <v>0</v>
       </c>
       <c r="R14" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
@@ -2863,17 +2733,14 @@
       <c r="D15" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>87</v>
+      <c r="E15" t="s">
+        <v>186</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
       <c r="G15" t="s">
-        <v>80</v>
-      </c>
-      <c r="H15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I15">
         <v>30008</v>
@@ -2900,7 +2767,7 @@
         <v>0</v>
       </c>
       <c r="R15" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
@@ -2908,25 +2775,22 @@
         <v>104011</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>82</v>
+      <c r="E16" t="s">
+        <v>187</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>78</v>
-      </c>
-      <c r="H16" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="I16">
         <v>30011</v>
@@ -2947,7 +2811,7 @@
         <v>0</v>
       </c>
       <c r="R16" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
@@ -2955,25 +2819,22 @@
         <v>104012</v>
       </c>
       <c r="B17" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>82</v>
+      <c r="E17" t="s">
+        <v>187</v>
       </c>
       <c r="F17">
         <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>78</v>
-      </c>
-      <c r="H17" t="s">
-        <v>115</v>
+        <v>68</v>
       </c>
       <c r="I17">
         <v>30012</v>
@@ -2994,7 +2855,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
@@ -3002,25 +2863,22 @@
         <v>104013</v>
       </c>
       <c r="B18" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>82</v>
+      <c r="E18" t="s">
+        <v>187</v>
       </c>
       <c r="F18">
         <v>3</v>
       </c>
       <c r="G18" t="s">
-        <v>78</v>
-      </c>
-      <c r="H18" t="s">
-        <v>116</v>
+        <v>68</v>
       </c>
       <c r="I18">
         <v>30013</v>
@@ -3041,7 +2899,7 @@
         <v>0</v>
       </c>
       <c r="R18" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
@@ -3049,25 +2907,22 @@
         <v>104021</v>
       </c>
       <c r="B19" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="C19" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="D19" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>82</v>
+      <c r="E19" t="s">
+        <v>188</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="G19" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="I19">
         <v>30011</v>
@@ -3094,7 +2949,7 @@
         <v>0</v>
       </c>
       <c r="R19" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
@@ -3102,25 +2957,22 @@
         <v>104022</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="D20" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>82</v>
+      <c r="E20" t="s">
+        <v>188</v>
       </c>
       <c r="F20">
         <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>80</v>
-      </c>
-      <c r="H20" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="I20">
         <v>30012</v>
@@ -3147,7 +2999,7 @@
         <v>0</v>
       </c>
       <c r="R20" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
@@ -3155,25 +3007,22 @@
         <v>104023</v>
       </c>
       <c r="B21" t="s">
-        <v>122</v>
+        <v>97</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D21" t="s">
         <v>14</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>82</v>
+      <c r="E21" t="s">
+        <v>188</v>
       </c>
       <c r="F21">
         <v>3</v>
       </c>
       <c r="G21" t="s">
-        <v>80</v>
-      </c>
-      <c r="H21" t="s">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="I21">
         <v>30013</v>
@@ -3200,7 +3049,7 @@
         <v>0</v>
       </c>
       <c r="R21" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
@@ -3208,25 +3057,22 @@
         <v>105011</v>
       </c>
       <c r="B22" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>82</v>
+      <c r="E22" t="s">
+        <v>189</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>78</v>
-      </c>
-      <c r="H22" t="s">
-        <v>117</v>
+        <v>68</v>
       </c>
       <c r="I22">
         <v>30016</v>
@@ -3247,7 +3093,7 @@
         <v>0</v>
       </c>
       <c r="R22" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
@@ -3255,25 +3101,22 @@
         <v>105012</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="C23" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>82</v>
+      <c r="E23" t="s">
+        <v>189</v>
       </c>
       <c r="F23">
         <v>2</v>
       </c>
       <c r="G23" t="s">
-        <v>78</v>
-      </c>
-      <c r="H23" t="s">
-        <v>117</v>
+        <v>68</v>
       </c>
       <c r="I23">
         <v>30017</v>
@@ -3294,7 +3137,7 @@
         <v>0</v>
       </c>
       <c r="R23" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
@@ -3302,25 +3145,22 @@
         <v>105013</v>
       </c>
       <c r="B24" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>82</v>
+      <c r="E24" t="s">
+        <v>189</v>
       </c>
       <c r="F24">
         <v>3</v>
       </c>
       <c r="G24" t="s">
-        <v>78</v>
-      </c>
-      <c r="H24" t="s">
-        <v>117</v>
+        <v>68</v>
       </c>
       <c r="I24">
         <v>30018</v>
@@ -3341,7 +3181,7 @@
         <v>0</v>
       </c>
       <c r="R24" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
@@ -3349,25 +3189,22 @@
         <v>105021</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="C25" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="D25" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>82</v>
+      <c r="E25" t="s">
+        <v>190</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>80</v>
-      </c>
-      <c r="H25" t="s">
-        <v>136</v>
+        <v>70</v>
       </c>
       <c r="I25">
         <v>30016</v>
@@ -3394,7 +3231,7 @@
         <v>0</v>
       </c>
       <c r="R25" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
@@ -3402,25 +3239,22 @@
         <v>105022</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="C26" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="D26" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>82</v>
+      <c r="E26" t="s">
+        <v>190</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
       <c r="G26" t="s">
-        <v>80</v>
-      </c>
-      <c r="H26" t="s">
-        <v>136</v>
+        <v>70</v>
       </c>
       <c r="I26">
         <v>30017</v>
@@ -3447,7 +3281,7 @@
         <v>0</v>
       </c>
       <c r="R26" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
@@ -3455,25 +3289,22 @@
         <v>105023</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="C27" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D27" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>82</v>
+      <c r="E27" t="s">
+        <v>190</v>
       </c>
       <c r="F27">
         <v>3</v>
       </c>
       <c r="G27" t="s">
-        <v>80</v>
-      </c>
-      <c r="H27" t="s">
-        <v>136</v>
+        <v>70</v>
       </c>
       <c r="I27">
         <v>30018</v>
@@ -3500,7 +3331,7 @@
         <v>0</v>
       </c>
       <c r="R27" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
@@ -3508,25 +3339,22 @@
         <v>106011</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="C28" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>82</v>
+      <c r="E28" t="s">
+        <v>191</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>78</v>
-      </c>
-      <c r="H28" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="I28">
         <v>30021</v>
@@ -3547,7 +3375,7 @@
         <v>0</v>
       </c>
       <c r="R28" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
@@ -3555,25 +3383,22 @@
         <v>106012</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="C29" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>82</v>
+      <c r="E29" t="s">
+        <v>191</v>
       </c>
       <c r="F29">
         <v>2</v>
       </c>
       <c r="G29" t="s">
-        <v>78</v>
-      </c>
-      <c r="H29" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="I29">
         <v>30022</v>
@@ -3594,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
@@ -3602,25 +3427,22 @@
         <v>106013</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C30" t="s">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>82</v>
+      <c r="E30" t="s">
+        <v>191</v>
       </c>
       <c r="F30">
         <v>3</v>
       </c>
       <c r="G30" t="s">
-        <v>78</v>
-      </c>
-      <c r="H30" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="I30">
         <v>30023</v>
@@ -3641,7 +3463,7 @@
         <v>0</v>
       </c>
       <c r="R30" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
@@ -3649,25 +3471,22 @@
         <v>106021</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C31" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
       <c r="D31" t="s">
         <v>14</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>82</v>
+      <c r="E31" t="s">
+        <v>192</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31" t="s">
-        <v>80</v>
-      </c>
-      <c r="H31" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="I31">
         <v>30021</v>
@@ -3694,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="R31" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
@@ -3702,25 +3521,22 @@
         <v>106022</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="C32" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="D32" t="s">
         <v>14</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>82</v>
+      <c r="E32" t="s">
+        <v>192</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H32" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="I32">
         <v>30022</v>
@@ -3747,7 +3563,7 @@
         <v>0</v>
       </c>
       <c r="R32" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.3">
@@ -3755,25 +3571,22 @@
         <v>106023</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="C33" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="D33" t="s">
         <v>14</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>82</v>
+      <c r="E33" t="s">
+        <v>192</v>
       </c>
       <c r="F33">
         <v>3</v>
       </c>
       <c r="G33" t="s">
-        <v>80</v>
-      </c>
-      <c r="H33" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="I33">
         <v>30023</v>
@@ -3800,7 +3613,7 @@
         <v>0</v>
       </c>
       <c r="R33" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.3">
@@ -3808,25 +3621,22 @@
         <v>107011</v>
       </c>
       <c r="B34" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="C34" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>82</v>
+      <c r="E34" t="s">
+        <v>193</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" t="s">
-        <v>78</v>
-      </c>
-      <c r="H34" t="s">
-        <v>150</v>
+        <v>68</v>
       </c>
       <c r="I34">
         <v>30026</v>
@@ -3847,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="R34" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.3">
@@ -3855,25 +3665,22 @@
         <v>107012</v>
       </c>
       <c r="B35" t="s">
-        <v>139</v>
+        <v>110</v>
       </c>
       <c r="C35" t="s">
-        <v>145</v>
+        <v>116</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>82</v>
+      <c r="E35" t="s">
+        <v>193</v>
       </c>
       <c r="F35">
         <v>2</v>
       </c>
       <c r="G35" t="s">
-        <v>78</v>
-      </c>
-      <c r="H35" t="s">
-        <v>150</v>
+        <v>68</v>
       </c>
       <c r="I35">
         <v>30027</v>
@@ -3894,7 +3701,7 @@
         <v>0</v>
       </c>
       <c r="R35" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.3">
@@ -3902,25 +3709,22 @@
         <v>107013</v>
       </c>
       <c r="B36" t="s">
-        <v>140</v>
+        <v>111</v>
       </c>
       <c r="C36" t="s">
-        <v>149</v>
+        <v>120</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>82</v>
+      <c r="E36" t="s">
+        <v>193</v>
       </c>
       <c r="F36">
         <v>3</v>
       </c>
       <c r="G36" t="s">
-        <v>78</v>
-      </c>
-      <c r="H36" t="s">
-        <v>150</v>
+        <v>68</v>
       </c>
       <c r="I36">
         <v>30028</v>
@@ -3941,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="R36" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.3">
@@ -3949,26 +3753,24 @@
         <v>107021</v>
       </c>
       <c r="B37" t="s">
-        <v>141</v>
+        <v>112</v>
       </c>
       <c r="C37" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
       <c r="D37" t="s">
         <v>14</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>82</v>
+      <c r="E37" t="s">
+        <v>194</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37" t="s">
-        <v>80</v>
-      </c>
-      <c r="H37" s="8" t="s">
-        <v>151</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H37" s="7"/>
       <c r="I37">
         <v>30026</v>
       </c>
@@ -3994,7 +3796,7 @@
         <v>0</v>
       </c>
       <c r="R37" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.3">
@@ -4002,26 +3804,24 @@
         <v>107022</v>
       </c>
       <c r="B38" t="s">
-        <v>142</v>
+        <v>113</v>
       </c>
       <c r="C38" t="s">
-        <v>147</v>
+        <v>118</v>
       </c>
       <c r="D38" t="s">
         <v>14</v>
       </c>
-      <c r="E38" s="2" t="s">
-        <v>82</v>
+      <c r="E38" t="s">
+        <v>194</v>
       </c>
       <c r="F38">
         <v>2</v>
       </c>
       <c r="G38" t="s">
-        <v>80</v>
-      </c>
-      <c r="H38" s="8" t="s">
-        <v>151</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H38" s="7"/>
       <c r="I38">
         <v>30027</v>
       </c>
@@ -4047,7 +3847,7 @@
         <v>0</v>
       </c>
       <c r="R38" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.3">
@@ -4055,26 +3855,24 @@
         <v>107023</v>
       </c>
       <c r="B39" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="C39" t="s">
-        <v>148</v>
+        <v>119</v>
       </c>
       <c r="D39" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="7" t="s">
-        <v>82</v>
+      <c r="E39" t="s">
+        <v>194</v>
       </c>
       <c r="F39">
         <v>3</v>
       </c>
       <c r="G39" t="s">
-        <v>80</v>
-      </c>
-      <c r="H39" s="8" t="s">
-        <v>151</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="H39" s="7"/>
       <c r="I39">
         <v>30028</v>
       </c>
@@ -4100,7 +3898,7 @@
         <v>0</v>
       </c>
       <c r="R39" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.3">
@@ -4108,25 +3906,25 @@
         <v>110001</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>39</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>89</v>
+        <v>57</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F40" s="4">
         <v>1</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
@@ -4144,7 +3942,7 @@
         <v>42</v>
       </c>
       <c r="R40" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.3">
@@ -4152,25 +3950,25 @@
         <v>110002</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>43</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F41" s="6">
         <v>2</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I41" s="6"/>
       <c r="J41" s="6">
@@ -4190,7 +3988,7 @@
         <v>42</v>
       </c>
       <c r="R41" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
@@ -4198,25 +3996,25 @@
         <v>110003</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>44</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F42" s="6">
         <v>3</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I42" s="6"/>
       <c r="J42" s="6">
@@ -4236,7 +4034,7 @@
         <v>42</v>
       </c>
       <c r="R42" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.3">
@@ -4244,25 +4042,25 @@
         <v>110004</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>45</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F43" s="6">
         <v>4</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I43" s="6"/>
       <c r="J43" s="6">
@@ -4282,7 +4080,7 @@
         <v>42</v>
       </c>
       <c r="R43" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
@@ -4290,25 +4088,25 @@
         <v>110005</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>187</v>
+        <v>155</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F44" s="6">
         <v>5</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I44" s="6"/>
       <c r="J44" s="6">
@@ -4328,7 +4126,7 @@
         <v>42</v>
       </c>
       <c r="R44" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.3">
@@ -4336,25 +4134,25 @@
         <v>110006</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>183</v>
+        <v>151</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F45" s="6">
         <v>6</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I45" s="6"/>
       <c r="J45" s="6">
@@ -4374,7 +4172,7 @@
         <v>42</v>
       </c>
       <c r="R45" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
@@ -4382,25 +4180,25 @@
         <v>110007</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="F46" s="6">
         <v>7</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I46" s="6"/>
       <c r="J46" s="6">
@@ -4420,7 +4218,7 @@
         <v>42</v>
       </c>
       <c r="R46" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.3">
@@ -4428,25 +4226,25 @@
         <v>111001</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>90</v>
+        <v>56</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F47" s="6">
         <v>1</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I47" s="6"/>
       <c r="J47" s="6"/>
@@ -4464,7 +4262,7 @@
         <v>42</v>
       </c>
       <c r="R47" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.3">
@@ -4472,25 +4270,25 @@
         <v>111002</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>90</v>
+        <v>56</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F48" s="4">
         <v>2</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I48" s="4"/>
       <c r="J48" s="6">
@@ -4510,7 +4308,7 @@
         <v>42</v>
       </c>
       <c r="R48" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.3">
@@ -4518,25 +4316,25 @@
         <v>111003</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>91</v>
+        <v>56</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F49" s="6">
         <v>3</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I49" s="6"/>
       <c r="J49" s="6">
@@ -4556,7 +4354,7 @@
         <v>42</v>
       </c>
       <c r="R49" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.3">
@@ -4564,25 +4362,25 @@
         <v>111004</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>92</v>
+        <v>56</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F50" s="4">
         <v>4</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I50" s="4"/>
       <c r="J50" s="6">
@@ -4602,7 +4400,7 @@
         <v>42</v>
       </c>
       <c r="R50" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.3">
@@ -4610,25 +4408,25 @@
         <v>111005</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C51" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D51" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>91</v>
+      <c r="E51" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F51" s="6">
         <v>5</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I51" s="6"/>
       <c r="J51" s="6">
@@ -4648,7 +4446,7 @@
         <v>42</v>
       </c>
       <c r="R51" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.3">
@@ -4656,25 +4454,25 @@
         <v>111006</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>171</v>
+        <v>140</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>172</v>
+        <v>141</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>90</v>
+        <v>56</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F52" s="6">
         <v>6</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I52" s="6"/>
       <c r="J52" s="6">
@@ -4694,7 +4492,7 @@
         <v>42</v>
       </c>
       <c r="R52" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.3">
@@ -4702,25 +4500,25 @@
         <v>111007</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>173</v>
+        <v>142</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>174</v>
+        <v>143</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>90</v>
+        <v>56</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="F53" s="6">
         <v>7</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I53" s="6"/>
       <c r="J53" s="6">
@@ -4740,7 +4538,7 @@
         <v>42</v>
       </c>
       <c r="R53" t="s">
-        <v>206</v>
+        <v>174</v>
       </c>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.3">
@@ -4748,31 +4546,31 @@
         <v>112001</v>
       </c>
       <c r="B54" t="s">
-        <v>175</v>
+        <v>144</v>
       </c>
       <c r="C54" t="s">
-        <v>165</v>
+        <v>134</v>
       </c>
       <c r="D54" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E54" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F54">
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H54" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="Q54" t="s">
         <v>0</v>
       </c>
       <c r="R54" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.3">
@@ -4780,25 +4578,25 @@
         <v>112002</v>
       </c>
       <c r="B55" t="s">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="C55" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="D55" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E55" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F55">
         <v>2</v>
       </c>
       <c r="G55" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H55" t="s">
-        <v>153</v>
+        <v>122</v>
       </c>
       <c r="I55">
         <v>30005</v>
@@ -4807,7 +4605,7 @@
         <v>0</v>
       </c>
       <c r="R55" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.3">
@@ -4815,25 +4613,25 @@
         <v>112003</v>
       </c>
       <c r="B56" t="s">
-        <v>155</v>
+        <v>124</v>
       </c>
       <c r="C56" t="s">
-        <v>166</v>
+        <v>135</v>
       </c>
       <c r="D56" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E56" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F56">
         <v>3</v>
       </c>
       <c r="G56" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H56" t="s">
-        <v>161</v>
+        <v>130</v>
       </c>
       <c r="I56">
         <v>30010</v>
@@ -4842,7 +4640,7 @@
         <v>0</v>
       </c>
       <c r="R56" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.3">
@@ -4850,25 +4648,25 @@
         <v>112004</v>
       </c>
       <c r="B57" t="s">
-        <v>156</v>
+        <v>125</v>
       </c>
       <c r="C57" t="s">
-        <v>167</v>
+        <v>136</v>
       </c>
       <c r="D57" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E57" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F57">
         <v>4</v>
       </c>
       <c r="G57" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H57" t="s">
-        <v>162</v>
+        <v>131</v>
       </c>
       <c r="I57">
         <v>30015</v>
@@ -4877,7 +4675,7 @@
         <v>0</v>
       </c>
       <c r="R57" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.3">
@@ -4885,25 +4683,25 @@
         <v>112005</v>
       </c>
       <c r="B58" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="C58" t="s">
-        <v>168</v>
+        <v>137</v>
       </c>
       <c r="D58" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E58" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F58">
         <v>5</v>
       </c>
       <c r="G58" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H58" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="I58">
         <v>30020</v>
@@ -4912,7 +4710,7 @@
         <v>0</v>
       </c>
       <c r="R58" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.3">
@@ -4920,25 +4718,25 @@
         <v>112006</v>
       </c>
       <c r="B59" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="C59" t="s">
-        <v>169</v>
+        <v>138</v>
       </c>
       <c r="D59" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E59" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F59">
         <v>6</v>
       </c>
       <c r="G59" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H59" t="s">
-        <v>164</v>
+        <v>133</v>
       </c>
       <c r="I59">
         <v>30025</v>
@@ -4947,7 +4745,7 @@
         <v>0</v>
       </c>
       <c r="R59" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.3">
@@ -4955,25 +4753,25 @@
         <v>112007</v>
       </c>
       <c r="B60" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="C60" t="s">
-        <v>170</v>
+        <v>139</v>
       </c>
       <c r="D60" t="s">
-        <v>176</v>
+        <v>145</v>
       </c>
       <c r="E60" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="F60">
         <v>7</v>
       </c>
       <c r="G60" t="s">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="H60" t="s">
-        <v>202</v>
+        <v>170</v>
       </c>
       <c r="I60">
         <v>30030</v>
@@ -4982,7 +4780,7 @@
         <v>0</v>
       </c>
       <c r="R60" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.3">
@@ -4990,25 +4788,25 @@
         <v>113001</v>
       </c>
       <c r="B61" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="C61" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="D61" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E61" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F61">
         <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H61" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="K61">
         <v>1002</v>
@@ -5020,7 +4818,7 @@
         <v>42</v>
       </c>
       <c r="R61" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.3">
@@ -5028,25 +4826,25 @@
         <v>113002</v>
       </c>
       <c r="B62" t="s">
-        <v>188</v>
+        <v>156</v>
       </c>
       <c r="C62" t="s">
-        <v>189</v>
+        <v>157</v>
       </c>
       <c r="D62" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E62" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F62">
         <v>2</v>
       </c>
       <c r="G62" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H62" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="J62" s="6">
         <v>2</v>
@@ -5061,7 +4859,7 @@
         <v>42</v>
       </c>
       <c r="R62" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.3">
@@ -5069,25 +4867,25 @@
         <v>113003</v>
       </c>
       <c r="B63" t="s">
-        <v>190</v>
+        <v>158</v>
       </c>
       <c r="C63" t="s">
-        <v>191</v>
+        <v>159</v>
       </c>
       <c r="D63" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E63" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F63">
         <v>3</v>
       </c>
       <c r="G63" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H63" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="J63" s="6">
         <v>3</v>
@@ -5099,10 +4897,10 @@
         <v>20000</v>
       </c>
       <c r="Q63" s="2" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="R63" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.3">
@@ -5110,25 +4908,25 @@
         <v>113004</v>
       </c>
       <c r="B64" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
       <c r="C64" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
       <c r="D64" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E64" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F64">
         <v>4</v>
       </c>
       <c r="G64" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H64" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="J64" s="6">
         <v>4</v>
@@ -5140,10 +4938,10 @@
         <v>20000</v>
       </c>
       <c r="Q64" s="2" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="R64" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.3">
@@ -5151,25 +4949,25 @@
         <v>113005</v>
       </c>
       <c r="B65" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="C65" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="D65" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E65" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F65">
         <v>5</v>
       </c>
       <c r="G65" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H65" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="J65" s="6">
         <v>5</v>
@@ -5181,10 +4979,10 @@
         <v>20000</v>
       </c>
       <c r="Q65" s="2" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="R65" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="66" spans="1:18" x14ac:dyDescent="0.3">
@@ -5192,25 +4990,25 @@
         <v>113006</v>
       </c>
       <c r="B66" t="s">
-        <v>196</v>
+        <v>164</v>
       </c>
       <c r="C66" t="s">
-        <v>197</v>
+        <v>165</v>
       </c>
       <c r="D66" t="s">
-        <v>210</v>
+        <v>177</v>
       </c>
       <c r="E66" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F66">
         <v>6</v>
       </c>
       <c r="G66" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H66" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="J66" s="6">
         <v>6</v>
@@ -5222,10 +5020,10 @@
         <v>20000</v>
       </c>
       <c r="Q66" s="2" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="R66" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.3">
@@ -5233,25 +5031,25 @@
         <v>113007</v>
       </c>
       <c r="B67" t="s">
+        <v>166</v>
+      </c>
+      <c r="C67" t="s">
+        <v>167</v>
+      </c>
+      <c r="D67" t="s">
+        <v>177</v>
+      </c>
+      <c r="E67" t="s">
         <v>198</v>
-      </c>
-      <c r="C67" t="s">
-        <v>199</v>
-      </c>
-      <c r="D67" t="s">
-        <v>210</v>
-      </c>
-      <c r="E67" t="s">
-        <v>209</v>
       </c>
       <c r="F67">
         <v>7</v>
       </c>
       <c r="G67" t="s">
-        <v>208</v>
+        <v>176</v>
       </c>
       <c r="H67" t="s">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="J67" s="6">
         <v>7</v>
@@ -5263,10 +5061,10 @@
         <v>20000</v>
       </c>
       <c r="Q67" s="2" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="R67" t="s">
-        <v>207</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>